<commit_message>
chore: refine grammar templates
- Adjusted grammar structures to improve sentence fluency
- Ensured templates generate more natural and contextually accurate outputs
- Increased consistency across rule engine examples
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/data/source_tables/transaction.xlsx
+++ b/Text2SQL_Template/data/source_tables/transaction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\intent\dtb-explain\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\data\source_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1423E45E-2E3C-4E6F-941B-5C493071463C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAD68D6-AB66-489F-90CE-F4578F77C619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1191" yWindow="1551" windowWidth="17563" windowHeight="12575" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tên cột" sheetId="1" r:id="rId1"/>
@@ -208,9 +208,6 @@
     <t>from_account_currency</t>
   </si>
   <si>
-    <t>Loại tiền tệ của tài khoản nguồn (VND, USD, EUR...).</t>
-  </si>
-  <si>
     <t>from_account_fullname</t>
   </si>
   <si>
@@ -592,9 +589,6 @@
     <t>bill_type</t>
   </si>
   <si>
-    <t>Loại hóa đơn (Điện, Nước, Internet, Truyền hình...).</t>
-  </si>
-  <si>
     <t>bill_code</t>
   </si>
   <si>
@@ -743,6 +737,12 @@
   </si>
   <si>
     <t>Mã CIF (Customer Information File) của người chuyển (tương tự from_cust_no nhưng thường dùng định danh Core Banking).</t>
+  </si>
+  <si>
+    <t>Loại hóa đơn (Điện, Nước, Internet, Truyền hình).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại tiền tệ của tài khoản nguồn </t>
   </si>
 </sst>
 </file>
@@ -1363,7 +1363,7 @@
         <v>61</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>62</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1371,10 +1371,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1382,10 +1382,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1393,10 +1393,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1404,10 +1404,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1415,10 +1415,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1426,10 +1426,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1437,10 +1437,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1448,10 +1448,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1459,10 +1459,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1470,10 +1470,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1481,10 +1481,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1492,10 +1492,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1503,10 +1503,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1514,10 +1514,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1525,10 +1525,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1536,10 +1536,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1547,10 +1547,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1558,10 +1558,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1569,10 +1569,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1580,10 +1580,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1591,10 +1591,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1602,10 +1602,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1613,10 +1613,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1624,10 +1624,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1635,10 +1635,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1646,10 +1646,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1657,10 +1657,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1668,10 +1668,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1679,10 +1679,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1690,10 +1690,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1701,10 +1701,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1712,10 +1712,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1723,10 +1723,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1734,10 +1734,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1745,10 +1745,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1756,10 +1756,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1767,10 +1767,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1778,10 +1778,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1789,10 +1789,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1800,10 +1800,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1811,10 +1811,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1822,10 +1822,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1833,10 +1833,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1844,10 +1844,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1855,10 +1855,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1866,10 +1866,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C77" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1877,10 +1877,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1888,10 +1888,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1899,10 +1899,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1910,10 +1910,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C81" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1921,10 +1921,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1932,10 +1932,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1943,10 +1943,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1954,10 +1954,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1965,10 +1965,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1976,10 +1976,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1987,10 +1987,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1998,10 +1998,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2009,10 +2009,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2020,10 +2020,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2031,10 +2031,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2042,10 +2042,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2053,10 +2053,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2064,10 +2064,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>190</v>
+        <v>239</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2075,10 +2075,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2086,10 +2086,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2097,10 +2097,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2108,10 +2108,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2119,10 +2119,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2130,10 +2130,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2141,10 +2141,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2152,10 +2152,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2163,10 +2163,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2174,10 +2174,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2185,10 +2185,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2196,10 +2196,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2207,10 +2207,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2218,10 +2218,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2229,10 +2229,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2240,10 +2240,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2251,10 +2251,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2262,10 +2262,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2273,10 +2273,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2284,10 +2284,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2295,10 +2295,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2306,10 +2306,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2317,10 +2317,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2328,10 +2328,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2339,10 +2339,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(generator): refine profiler description handling for keyword filtering
- Improved description processing logic within profiler
- Added keyword filtering to enhance contextual accuracy
- Optimized integration with generator module for cleaner and more relevant outputs
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/data/source_tables/transaction.xlsx
+++ b/Text2SQL_Template/data/source_tables/transaction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\data\source_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAD68D6-AB66-489F-90CE-F4578F77C619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70185913-C453-4015-964A-C74F9ACA727B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,9 +64,6 @@
     <t>user_id</t>
   </si>
   <si>
-    <t>Mã định danh (ID) của người dùng thực hiện giao dịch (thường là khóa ngoại trỏ sang bảng User).</t>
-  </si>
-  <si>
     <t>user_name</t>
   </si>
   <si>
@@ -743,6 +740,9 @@
   </si>
   <si>
     <t xml:space="preserve">Loại tiền tệ của tài khoản nguồn </t>
+  </si>
+  <si>
+    <t>Mã định danh của người dùng thực hiện giao dịch (thường là khóa ngoại trỏ sang bảng User).</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1099,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>14</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1107,10 +1107,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1118,10 +1118,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1129,10 +1129,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1140,10 +1140,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1151,10 +1151,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1162,10 +1162,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1173,10 +1173,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1184,10 +1184,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1195,10 +1195,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1206,10 +1206,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1217,10 +1217,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1228,10 +1228,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1239,10 +1239,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1250,10 +1250,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1261,10 +1261,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1272,10 +1272,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1283,10 +1283,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1294,10 +1294,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1305,10 +1305,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1316,10 +1316,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1327,10 +1327,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1338,10 +1338,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1349,10 +1349,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1360,10 +1360,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1371,10 +1371,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1382,10 +1382,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1393,10 +1393,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1404,10 +1404,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1415,10 +1415,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1426,10 +1426,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1437,10 +1437,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1448,10 +1448,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1459,10 +1459,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1470,10 +1470,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1481,10 +1481,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1492,10 +1492,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1503,10 +1503,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1514,10 +1514,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1525,10 +1525,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1536,10 +1536,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1547,10 +1547,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1558,10 +1558,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1569,10 +1569,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1580,10 +1580,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1591,10 +1591,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1602,10 +1602,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1613,10 +1613,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1624,10 +1624,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1635,10 +1635,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1646,10 +1646,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1657,10 +1657,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1668,10 +1668,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1679,10 +1679,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1690,10 +1690,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1701,10 +1701,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1712,10 +1712,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1723,10 +1723,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1734,10 +1734,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1745,10 +1745,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1756,10 +1756,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1767,10 +1767,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1778,10 +1778,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1789,10 +1789,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1800,10 +1800,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1811,10 +1811,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1822,10 +1822,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1833,10 +1833,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>146</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1844,10 +1844,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1855,10 +1855,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1866,10 +1866,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C77" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1877,10 +1877,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1888,10 +1888,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1899,10 +1899,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1910,10 +1910,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C81" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1921,10 +1921,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1932,10 +1932,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1943,10 +1943,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1954,10 +1954,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1965,10 +1965,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1976,10 +1976,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1987,10 +1987,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -1998,10 +1998,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2009,10 +2009,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2020,10 +2020,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2031,10 +2031,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2042,10 +2042,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2053,10 +2053,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2064,10 +2064,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2075,10 +2075,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2086,10 +2086,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C97" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2097,10 +2097,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2108,10 +2108,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2119,10 +2119,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2130,10 +2130,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2141,10 +2141,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2152,10 +2152,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2163,10 +2163,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>205</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2174,10 +2174,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C105" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2185,10 +2185,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C106" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2196,10 +2196,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C107" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2207,10 +2207,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C108" s="1" t="s">
         <v>213</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2218,10 +2218,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2229,10 +2229,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C110" s="1" t="s">
         <v>217</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2240,10 +2240,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2251,10 +2251,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C112" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2262,10 +2262,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2273,10 +2273,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C114" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2284,10 +2284,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2295,10 +2295,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2306,10 +2306,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C117" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2317,10 +2317,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C118" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2328,10 +2328,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="12.45" x14ac:dyDescent="0.3">
@@ -2339,10 +2339,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C120" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>